<commit_message>
hotfix: add 625zz bearings to BOM
</commit_message>
<xml_diff>
--- a/Slipstream BOM.xlsx
+++ b/Slipstream BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaron/github/slipstream/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACA59837-B590-F74F-917A-C473D50097DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{638F472F-A655-5944-ADFF-742457E59A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39560" yWindow="5000" windowWidth="28040" windowHeight="23240" xr2:uid="{1A20C3FE-12CA-CF4E-93FC-B4FB38CAC438}"/>
+    <workbookView xWindow="31340" yWindow="2580" windowWidth="28040" windowHeight="23240" xr2:uid="{1A20C3FE-12CA-CF4E-93FC-B4FB38CAC438}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="100">
   <si>
     <t>Part Name</t>
   </si>
@@ -333,6 +333,9 @@
   </si>
   <si>
     <t>2020 90 Degree Frame Block 12x</t>
+  </si>
+  <si>
+    <t>625zz Bearing 25pcs</t>
   </si>
 </sst>
 </file>
@@ -782,7 +785,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{190AB665-411E-DC49-8B59-B2BCDE3E83A5}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:G88"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1026,7 +1029,7 @@
         <v>16.59</v>
       </c>
       <c r="E16" s="8">
-        <f t="shared" ref="E16:E29" si="1">PRODUCT(C16,D16)</f>
+        <f t="shared" ref="E16:E30" si="1">PRODUCT(C16,D16)</f>
         <v>16.59</v>
       </c>
       <c r="F16" s="5" t="b">
@@ -1110,17 +1113,17 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="C21">
         <v>1</v>
       </c>
       <c r="D21" s="8">
-        <v>8.99</v>
+        <v>7.79</v>
       </c>
       <c r="E21" s="8">
         <f t="shared" si="1"/>
-        <v>8.99</v>
+        <v>7.79</v>
       </c>
       <c r="F21" s="5" t="b">
         <v>0</v>
@@ -1128,17 +1131,17 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B22" s="7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C22">
         <v>1</v>
       </c>
       <c r="D22" s="8">
-        <v>40.99</v>
+        <v>8.99</v>
       </c>
       <c r="E22" s="8">
         <f t="shared" si="1"/>
-        <v>40.99</v>
+        <v>8.99</v>
       </c>
       <c r="F22" s="5" t="b">
         <v>0</v>
@@ -1146,17 +1149,17 @@
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B23" s="7" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
       <c r="D23" s="8">
-        <v>32.99</v>
+        <v>40.99</v>
       </c>
       <c r="E23" s="8">
         <f t="shared" si="1"/>
-        <v>32.99</v>
+        <v>40.99</v>
       </c>
       <c r="F23" s="5" t="b">
         <v>0</v>
@@ -1164,17 +1167,17 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B24" s="7" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C24">
         <v>1</v>
       </c>
       <c r="D24" s="8">
-        <v>25.99</v>
+        <v>32.99</v>
       </c>
       <c r="E24" s="8">
         <f t="shared" si="1"/>
-        <v>25.99</v>
+        <v>32.99</v>
       </c>
       <c r="F24" s="5" t="b">
         <v>0</v>
@@ -1182,17 +1185,17 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B25" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C25">
         <v>1</v>
       </c>
       <c r="D25" s="8">
-        <v>12.98</v>
+        <v>25.99</v>
       </c>
       <c r="E25" s="8">
         <f t="shared" si="1"/>
-        <v>12.98</v>
+        <v>25.99</v>
       </c>
       <c r="F25" s="5" t="b">
         <v>0</v>
@@ -1200,17 +1203,17 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B26" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
       <c r="D26" s="8">
-        <v>13.98</v>
+        <v>12.98</v>
       </c>
       <c r="E26" s="8">
         <f t="shared" si="1"/>
-        <v>13.98</v>
+        <v>12.98</v>
       </c>
       <c r="F26" s="5" t="b">
         <v>0</v>
@@ -1218,353 +1221,350 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B27" s="7" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="C27">
         <v>1</v>
       </c>
       <c r="D27" s="8">
-        <v>8.49</v>
+        <v>13.98</v>
       </c>
       <c r="E27" s="8">
         <f t="shared" si="1"/>
-        <v>8.49</v>
+        <v>13.98</v>
       </c>
       <c r="F27" s="5" t="b">
         <v>0</v>
-      </c>
-      <c r="G27" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B28" s="7" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
       <c r="D28" s="8">
-        <v>7.99</v>
+        <v>8.49</v>
       </c>
       <c r="E28" s="8">
         <f t="shared" si="1"/>
-        <v>7.99</v>
+        <v>8.49</v>
       </c>
       <c r="F28" s="5" t="b">
         <v>0</v>
+      </c>
+      <c r="G28" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B29" s="7" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" s="8">
-        <v>6.99</v>
+        <v>7.99</v>
       </c>
       <c r="E29" s="8">
         <f t="shared" si="1"/>
+        <v>7.99</v>
+      </c>
+      <c r="F29" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B30" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30">
+        <v>1</v>
+      </c>
+      <c r="D30" s="8">
         <v>6.99</v>
       </c>
-      <c r="F29" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="2" t="s">
+      <c r="E30" s="8">
+        <f t="shared" si="1"/>
+        <v>6.99</v>
+      </c>
+      <c r="F30" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C31" s="2">
-        <v>1</v>
-      </c>
-      <c r="D31" s="9">
-        <v>31.26</v>
-      </c>
-      <c r="E31" s="9">
-        <f t="shared" ref="E31:E37" si="2">PRODUCT(C31,D31)</f>
-        <v>31.26</v>
-      </c>
-      <c r="F31" s="6" t="b">
-        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B32" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C32" s="2">
+        <v>1</v>
+      </c>
+      <c r="D32" s="9">
+        <v>31.26</v>
+      </c>
+      <c r="E32" s="9">
+        <f t="shared" ref="E32:E38" si="2">PRODUCT(C32,D32)</f>
+        <v>31.26</v>
+      </c>
+      <c r="F32" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C32" s="2">
-        <v>1</v>
-      </c>
-      <c r="D32" s="9">
+      <c r="C33" s="2">
+        <v>1</v>
+      </c>
+      <c r="D33" s="9">
         <v>28.54</v>
       </c>
-      <c r="E32" s="9">
+      <c r="E33" s="9">
         <f t="shared" si="2"/>
         <v>28.54</v>
       </c>
-      <c r="F32" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="4" t="s">
+      <c r="F33" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C33" s="2">
-        <v>1</v>
-      </c>
-      <c r="D33" s="9">
+      <c r="C34" s="2">
+        <v>1</v>
+      </c>
+      <c r="D34" s="9">
         <v>129.99</v>
       </c>
-      <c r="E33" s="9">
+      <c r="E34" s="9">
         <f t="shared" si="2"/>
         <v>129.99</v>
       </c>
-      <c r="F33" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B34" s="4" t="s">
+      <c r="F34" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C34" s="2">
-        <v>1</v>
-      </c>
-      <c r="D34" s="9">
+      <c r="C35" s="2">
+        <v>1</v>
+      </c>
+      <c r="D35" s="9">
         <v>50</v>
       </c>
-      <c r="E34" s="9">
+      <c r="E35" s="9">
         <f t="shared" si="2"/>
         <v>50</v>
       </c>
-      <c r="F34" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B35" s="4" t="s">
+      <c r="F35" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B36" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C35" s="2">
-        <v>1</v>
-      </c>
-      <c r="D35" s="9">
+      <c r="C36" s="2">
+        <v>1</v>
+      </c>
+      <c r="D36" s="9">
         <v>8.99</v>
       </c>
-      <c r="E35" s="9">
+      <c r="E36" s="9">
         <f t="shared" si="2"/>
         <v>8.99</v>
       </c>
-      <c r="F35" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B36" s="4" t="s">
+      <c r="F36" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B37" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C36" s="2">
-        <v>1</v>
-      </c>
-      <c r="D36" s="9">
+      <c r="C37" s="2">
+        <v>1</v>
+      </c>
+      <c r="D37" s="9">
         <v>39.99</v>
       </c>
-      <c r="E36" s="9">
+      <c r="E37" s="9">
         <f t="shared" si="2"/>
         <v>39.99</v>
       </c>
-      <c r="F36" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B37" s="4" t="s">
+      <c r="F37" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B38" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C37" s="2">
-        <v>1</v>
-      </c>
-      <c r="D37" s="9">
+      <c r="C38" s="2">
+        <v>1</v>
+      </c>
+      <c r="D38" s="9">
         <v>15</v>
       </c>
-      <c r="E37" s="9">
+      <c r="E38" s="9">
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="F37" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+      <c r="F38" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
         <v>22</v>
       </c>
-      <c r="D38" s="1"/>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B39" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C39">
-        <v>4</v>
-      </c>
-      <c r="D39" s="8">
-        <v>12.99</v>
-      </c>
-      <c r="E39" s="8">
-        <f t="shared" ref="E39:E45" si="3">PRODUCT(C39,D39)</f>
-        <v>51.96</v>
-      </c>
-      <c r="F39" s="5" t="b">
-        <v>0</v>
-      </c>
+      <c r="D39" s="1"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B40" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C40">
         <v>4</v>
       </c>
       <c r="D40" s="8">
+        <v>12.99</v>
+      </c>
+      <c r="E40" s="8">
+        <f t="shared" ref="E40:E46" si="3">PRODUCT(C40,D40)</f>
+        <v>51.96</v>
+      </c>
+      <c r="F40" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B41" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41">
+        <v>4</v>
+      </c>
+      <c r="D41" s="8">
         <v>15.6</v>
       </c>
-      <c r="E40" s="8">
+      <c r="E41" s="8">
         <f t="shared" si="3"/>
         <v>62.4</v>
       </c>
-      <c r="F40" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B41" s="7" t="s">
+      <c r="F41" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B42" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C41">
-        <v>1</v>
-      </c>
-      <c r="D41" s="8">
+      <c r="C42">
+        <v>1</v>
+      </c>
+      <c r="D42" s="8">
         <v>6.99</v>
       </c>
-      <c r="E41" s="8">
+      <c r="E42" s="8">
         <f t="shared" si="3"/>
         <v>6.99</v>
       </c>
-      <c r="F41" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B42" s="7" t="s">
+      <c r="F42" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B43" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C42">
-        <v>1</v>
-      </c>
-      <c r="D42" s="8">
+      <c r="C43">
+        <v>1</v>
+      </c>
+      <c r="D43" s="8">
         <v>13.99</v>
       </c>
-      <c r="E42" s="8">
+      <c r="E43" s="8">
         <f t="shared" si="3"/>
         <v>13.99</v>
       </c>
-      <c r="F42" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="2" t="s">
+      <c r="F43" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B44" s="4" t="s">
+    <row r="45" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B45" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C44" s="2">
-        <v>1</v>
-      </c>
-      <c r="D44" s="9">
+      <c r="C45" s="2">
+        <v>1</v>
+      </c>
+      <c r="D45" s="9">
         <v>22.99</v>
       </c>
-      <c r="E44" s="9">
+      <c r="E45" s="9">
         <f t="shared" si="3"/>
         <v>22.99</v>
       </c>
-      <c r="F44" s="6" t="b">
-        <v>0</v>
-      </c>
-      <c r="G44" s="4" t="s">
+      <c r="F45" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G45" s="4" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="45" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B45" s="4" t="s">
+    <row r="46" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B46" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C45" s="2">
-        <v>1</v>
-      </c>
-      <c r="D45" s="9">
+      <c r="C46" s="2">
+        <v>1</v>
+      </c>
+      <c r="D46" s="9">
         <v>12.99</v>
       </c>
-      <c r="E45" s="9">
+      <c r="E46" s="9">
         <f t="shared" si="3"/>
         <v>12.99</v>
       </c>
-      <c r="F45" s="6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+      <c r="F46" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B47" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C47">
-        <v>1</v>
-      </c>
-      <c r="D47" s="8">
-        <v>7.59</v>
-      </c>
-      <c r="E47" s="8">
-        <f>PRODUCT(C47,D47)</f>
-        <v>7.59</v>
-      </c>
-      <c r="F47" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G47" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B48" s="7" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="C48">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D48" s="8">
-        <v>11.99</v>
+        <v>7.59</v>
       </c>
       <c r="E48" s="8">
         <f>PRODUCT(C48,D48)</f>
-        <v>23.98</v>
+        <v>7.59</v>
       </c>
       <c r="F48" s="5" t="b">
         <v>0</v>
@@ -1575,17 +1575,17 @@
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B49" s="7" t="s">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="C49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D49" s="8">
-        <v>7.99</v>
+        <v>11.99</v>
       </c>
       <c r="E49" s="8">
         <f>PRODUCT(C49,D49)</f>
-        <v>7.99</v>
+        <v>23.98</v>
       </c>
       <c r="F49" s="5" t="b">
         <v>0</v>
@@ -1596,75 +1596,88 @@
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B50" s="7" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="C50">
         <v>1</v>
       </c>
       <c r="D50" s="8">
-        <v>9.99</v>
+        <v>7.99</v>
       </c>
       <c r="E50" s="8">
         <f>PRODUCT(C50,D50)</f>
-        <v>9.99</v>
+        <v>7.99</v>
       </c>
       <c r="F50" s="5" t="b">
         <v>0</v>
+      </c>
+      <c r="G50" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B51" s="7" t="s">
-        <v>96</v>
+        <v>34</v>
       </c>
       <c r="C51">
         <v>1</v>
       </c>
       <c r="D51" s="8">
-        <v>14.49</v>
+        <v>9.99</v>
       </c>
       <c r="E51" s="8">
         <f>PRODUCT(C51,D51)</f>
+        <v>9.99</v>
+      </c>
+      <c r="F51" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B52" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C52">
+        <v>1</v>
+      </c>
+      <c r="D52" s="8">
         <v>14.49</v>
       </c>
-      <c r="F51" s="5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="2" t="s">
+      <c r="E52" s="8">
+        <f>PRODUCT(C52,D52)</f>
+        <v>14.49</v>
+      </c>
+      <c r="F52" s="5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B52" s="10" t="s">
+      <c r="B53" s="10" t="s">
         <v>91</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B53" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C53" s="2">
-        <v>16</v>
       </c>
     </row>
     <row r="54" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B54" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C54" s="2">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="55" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B55" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C55" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B56" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C56" s="2">
         <v>8</v>
@@ -1672,7 +1685,7 @@
     </row>
     <row r="57" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B57" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C57" s="2">
         <v>8</v>
@@ -1680,220 +1693,228 @@
     </row>
     <row r="58" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B58" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C58" s="2">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="59" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B59" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C59" s="2">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="60" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B60" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C60" s="2">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="61" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B61" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C61" s="2">
-        <v>56</v>
+        <v>8</v>
       </c>
     </row>
     <row r="62" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B62" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C62" s="2">
-        <v>8</v>
+        <v>56</v>
       </c>
     </row>
     <row r="63" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B63" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C63" s="2">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="64" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B64" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C64" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B65" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C65" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="66" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B66" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C66" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B67" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C67" s="2">
-        <v>28</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B68" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C68" s="2">
-        <v>5</v>
+        <v>28</v>
       </c>
     </row>
     <row r="69" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B69" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C69" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B70" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C70" s="2">
-        <v>42</v>
+        <v>6</v>
       </c>
     </row>
     <row r="71" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B71" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C71" s="2">
-        <v>24</v>
+        <v>42</v>
       </c>
     </row>
     <row r="72" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B72" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C72" s="2">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="73" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B73" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C73" s="2">
-        <v>108</v>
+        <v>16</v>
       </c>
     </row>
     <row r="74" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B74" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C74" s="2">
-        <v>6</v>
+        <v>108</v>
       </c>
     </row>
     <row r="75" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B75" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C75" s="2">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B76" s="2" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C76" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="77" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B77" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C77" s="2">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="78" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B78" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C78" s="2">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="79" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B79" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C79" s="2">
-        <v>32</v>
+        <v>5</v>
       </c>
     </row>
     <row r="80" spans="2:3" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B80" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C80" s="2">
-        <v>41</v>
+        <v>32</v>
       </c>
     </row>
     <row r="81" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B81" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C81" s="2">
-        <v>3</v>
+        <v>41</v>
       </c>
     </row>
     <row r="82" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="B82" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C82" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="83" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B83" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C82" s="2">
+      <c r="C83" s="2">
         <v>18</v>
-      </c>
-    </row>
-    <row r="87" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="D87" t="s">
-        <v>24</v>
-      </c>
-      <c r="E87" s="8">
-        <f>SUM(E3:E50)</f>
-        <v>1414.0200000000002</v>
       </c>
     </row>
     <row r="88" spans="2:5" x14ac:dyDescent="0.2">
       <c r="D88" t="s">
+        <v>24</v>
+      </c>
+      <c r="E88" s="8">
+        <f>SUM(E3:E51)</f>
+        <v>1421.8100000000002</v>
+      </c>
+    </row>
+    <row r="89" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="D89" t="s">
         <v>25</v>
       </c>
-      <c r="E88" s="8">
-        <f>E87-SUMIFS(E3:E50, F3:F50, TRUE)</f>
-        <v>1414.0200000000002</v>
+      <c r="E89" s="8">
+        <f>E88-SUMIFS(E3:E51, F3:F51, TRUE)</f>
+        <v>1421.8100000000002</v>
       </c>
     </row>
   </sheetData>
@@ -1910,36 +1931,37 @@
     <hyperlink ref="B17" r:id="rId10" xr:uid="{8EE96F24-63A2-9B4E-AD9C-72620609C969}"/>
     <hyperlink ref="B18" r:id="rId11" xr:uid="{E559603D-F3D2-174F-A94A-47CA4046C818}"/>
     <hyperlink ref="B19" r:id="rId12" display="MGN12H 350MM" xr:uid="{223BCBA6-86A9-2144-8F2C-75C9B68057A0}"/>
-    <hyperlink ref="B21" r:id="rId13" xr:uid="{D8513075-F571-2C4B-95FA-1016C3C29CEE}"/>
-    <hyperlink ref="B22" r:id="rId14" xr:uid="{3FFBA4CD-8F94-EE42-B36C-B1CC4968A446}"/>
-    <hyperlink ref="B23" r:id="rId15" xr:uid="{D57C98A0-3DAC-7C4D-90F4-7BD33AEF0B08}"/>
-    <hyperlink ref="B24" r:id="rId16" xr:uid="{9464945C-9434-F94D-9B05-F9F116CDF1BB}"/>
-    <hyperlink ref="B25" r:id="rId17" xr:uid="{8DB43896-FA61-0A47-9375-98EEB379F425}"/>
-    <hyperlink ref="B26" r:id="rId18" xr:uid="{841DF760-DB22-B248-AF7E-21C6498CC9EE}"/>
-    <hyperlink ref="B27" r:id="rId19" xr:uid="{8D0DD199-FCDD-BE4C-8428-62EEC2391CD4}"/>
-    <hyperlink ref="B28" r:id="rId20" xr:uid="{B2A7B9FB-F184-3643-A1E3-1A39F55CB90F}"/>
-    <hyperlink ref="B29" r:id="rId21" xr:uid="{D71855D8-9C7C-4841-9CF0-F3F6EDA6947F}"/>
-    <hyperlink ref="B31" r:id="rId22" xr:uid="{F2098D89-359C-7B46-B857-24FDB225BC5C}"/>
-    <hyperlink ref="B32" r:id="rId23" xr:uid="{D9FA7A25-2ABB-A348-9EAA-6A0BD7AC274A}"/>
-    <hyperlink ref="B33" r:id="rId24" xr:uid="{ADF328AB-1FC0-EF44-AE87-5623AF89980A}"/>
-    <hyperlink ref="B34" r:id="rId25" xr:uid="{A14C6C7F-568D-6B44-985D-3F56EC4114E5}"/>
-    <hyperlink ref="B35" r:id="rId26" xr:uid="{2A305941-7ADB-1B4B-A74E-A642B558D874}"/>
-    <hyperlink ref="B36" r:id="rId27" xr:uid="{BDC9F487-FCC2-A348-A761-8BD99493C513}"/>
-    <hyperlink ref="B37" r:id="rId28" xr:uid="{988EFBD5-F8D7-8548-A6D9-39C452C56754}"/>
-    <hyperlink ref="B39" r:id="rId29" xr:uid="{E8C38802-504C-C349-926C-8B88345343A7}"/>
-    <hyperlink ref="B40" r:id="rId30" xr:uid="{1D4F1698-43C2-F743-9931-BE4792783BF3}"/>
-    <hyperlink ref="B41" r:id="rId31" xr:uid="{1C2B42C2-8289-9B46-98D8-1A365CDC6E78}"/>
-    <hyperlink ref="B42" r:id="rId32" xr:uid="{3E30D6F6-C1DA-8E4F-BBD5-0E83580163D5}"/>
-    <hyperlink ref="B44" r:id="rId33" xr:uid="{32765079-8A55-E145-8E73-CD39487A166B}"/>
-    <hyperlink ref="B45" r:id="rId34" xr:uid="{B14474BD-C9E7-DE4A-9C73-4B99DF8F334B}"/>
-    <hyperlink ref="B47" r:id="rId35" xr:uid="{FC871B89-1511-C64D-97C7-92774D760E18}"/>
-    <hyperlink ref="B48" r:id="rId36" display="M3 heat inserts 500ct" xr:uid="{ED1CE362-166F-FE48-87E8-AA349BB642C2}"/>
-    <hyperlink ref="B49" r:id="rId37" xr:uid="{0FA132B0-22D4-6B46-A5F1-39C8708362AA}"/>
-    <hyperlink ref="B50" r:id="rId38" xr:uid="{C816B0DB-70B2-0940-A4A6-8E45792C06B1}"/>
-    <hyperlink ref="G44" r:id="rId39" display="Nicer option here" xr:uid="{19AD8014-89EF-0E4F-AE22-5CAE74DBE606}"/>
+    <hyperlink ref="B22" r:id="rId13" xr:uid="{D8513075-F571-2C4B-95FA-1016C3C29CEE}"/>
+    <hyperlink ref="B23" r:id="rId14" xr:uid="{3FFBA4CD-8F94-EE42-B36C-B1CC4968A446}"/>
+    <hyperlink ref="B24" r:id="rId15" xr:uid="{D57C98A0-3DAC-7C4D-90F4-7BD33AEF0B08}"/>
+    <hyperlink ref="B25" r:id="rId16" xr:uid="{9464945C-9434-F94D-9B05-F9F116CDF1BB}"/>
+    <hyperlink ref="B26" r:id="rId17" xr:uid="{8DB43896-FA61-0A47-9375-98EEB379F425}"/>
+    <hyperlink ref="B27" r:id="rId18" xr:uid="{841DF760-DB22-B248-AF7E-21C6498CC9EE}"/>
+    <hyperlink ref="B28" r:id="rId19" xr:uid="{8D0DD199-FCDD-BE4C-8428-62EEC2391CD4}"/>
+    <hyperlink ref="B29" r:id="rId20" xr:uid="{B2A7B9FB-F184-3643-A1E3-1A39F55CB90F}"/>
+    <hyperlink ref="B30" r:id="rId21" xr:uid="{D71855D8-9C7C-4841-9CF0-F3F6EDA6947F}"/>
+    <hyperlink ref="B32" r:id="rId22" xr:uid="{F2098D89-359C-7B46-B857-24FDB225BC5C}"/>
+    <hyperlink ref="B33" r:id="rId23" xr:uid="{D9FA7A25-2ABB-A348-9EAA-6A0BD7AC274A}"/>
+    <hyperlink ref="B34" r:id="rId24" xr:uid="{ADF328AB-1FC0-EF44-AE87-5623AF89980A}"/>
+    <hyperlink ref="B35" r:id="rId25" xr:uid="{A14C6C7F-568D-6B44-985D-3F56EC4114E5}"/>
+    <hyperlink ref="B36" r:id="rId26" xr:uid="{2A305941-7ADB-1B4B-A74E-A642B558D874}"/>
+    <hyperlink ref="B37" r:id="rId27" xr:uid="{BDC9F487-FCC2-A348-A761-8BD99493C513}"/>
+    <hyperlink ref="B38" r:id="rId28" xr:uid="{988EFBD5-F8D7-8548-A6D9-39C452C56754}"/>
+    <hyperlink ref="B40" r:id="rId29" xr:uid="{E8C38802-504C-C349-926C-8B88345343A7}"/>
+    <hyperlink ref="B41" r:id="rId30" xr:uid="{1D4F1698-43C2-F743-9931-BE4792783BF3}"/>
+    <hyperlink ref="B42" r:id="rId31" xr:uid="{1C2B42C2-8289-9B46-98D8-1A365CDC6E78}"/>
+    <hyperlink ref="B43" r:id="rId32" xr:uid="{3E30D6F6-C1DA-8E4F-BBD5-0E83580163D5}"/>
+    <hyperlink ref="B45" r:id="rId33" xr:uid="{32765079-8A55-E145-8E73-CD39487A166B}"/>
+    <hyperlink ref="B46" r:id="rId34" xr:uid="{B14474BD-C9E7-DE4A-9C73-4B99DF8F334B}"/>
+    <hyperlink ref="B48" r:id="rId35" xr:uid="{FC871B89-1511-C64D-97C7-92774D760E18}"/>
+    <hyperlink ref="B49" r:id="rId36" display="M3 heat inserts 500ct" xr:uid="{ED1CE362-166F-FE48-87E8-AA349BB642C2}"/>
+    <hyperlink ref="B50" r:id="rId37" xr:uid="{0FA132B0-22D4-6B46-A5F1-39C8708362AA}"/>
+    <hyperlink ref="B51" r:id="rId38" xr:uid="{C816B0DB-70B2-0940-A4A6-8E45792C06B1}"/>
+    <hyperlink ref="G45" r:id="rId39" display="Nicer option here" xr:uid="{19AD8014-89EF-0E4F-AE22-5CAE74DBE606}"/>
     <hyperlink ref="B20" r:id="rId40" xr:uid="{426B2FB9-0E94-9649-B1BB-038564564347}"/>
-    <hyperlink ref="B51" r:id="rId41" xr:uid="{FC1CC4D9-5B92-E746-AED6-8B6B2A9B2F4B}"/>
+    <hyperlink ref="B52" r:id="rId41" xr:uid="{FC1CC4D9-5B92-E746-AED6-8B6B2A9B2F4B}"/>
     <hyperlink ref="B14" r:id="rId42" xr:uid="{538BF64F-4CCC-F349-882A-A7E2A969C667}"/>
+    <hyperlink ref="B21" r:id="rId43" xr:uid="{AF4FC672-4EFE-B04D-BB09-F9AE1119DBC3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>